<commit_message>
Fix beta sample: complete every group with IPCC catalogue defaults
The sample supplied only a subset of parameters per sub-category. The app's
template writer emits one Parameters row per catalogue parameter per group but
only pre-fills the FIRST group's gaps (from the blank-template skeleton); groups
2+ came through with blank value/distribution cells, so upload failed with
"Invalid distribution: Fat, Cfi, Ca, C, Cp, ...".

_make_sample_inventory.R now backfills each group's unset parameters with the
PARAM_CATALOGUE default value / distribution / uncertainty (data_source =
"ipcc_default") — asymmetric params take the catalogue's explicit lower/upper
bounds, symmetric ones derive bounds from mean ± uncertainty%. This mirrors a
complete inventory / AI-translator output.

Regenerated beta_sample_inventory.xlsx: 100 parameter rows (25 x 4 groups),
no blank distributions; validate_param_specs() returns valid = TRUE, no errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feedback_workflow/beta_sample_inventory.xlsx
+++ b/feedback_workflow/beta_sample_inventory.xlsx
@@ -3534,7 +3534,7 @@
         <v>203</v>
       </c>
       <c r="P12" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
@@ -3580,7 +3580,7 @@
         <v>207</v>
       </c>
       <c r="P13" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -3626,7 +3626,7 @@
         <v>210</v>
       </c>
       <c r="P14" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -3672,7 +3672,7 @@
         <v>213</v>
       </c>
       <c r="P15" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -3694,7 +3694,9 @@
       <c r="F16" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="G16" s="3"/>
+      <c r="G16" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="H16" s="3" t="n">
         <v>20</v>
       </c>
@@ -3703,11 +3705,11 @@
       <c r="K16" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L16" s="6" t="str">
-        <f>=IF(I16&lt;&gt;"",I16,IF(AND(G16&lt;&gt;"",H16&lt;&gt;""),G16*(1-H16/100),""))</f>
-      </c>
-      <c r="M16" s="6" t="str">
-        <f>=IF(J16&lt;&gt;"",J16,IF(AND(G16&lt;&gt;"",H16&lt;&gt;""),G16*(1+H16/100),""))</f>
+      <c r="L16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="N16" s="5" t="s">
         <v>15</v>
@@ -3716,7 +3718,7 @@
         <v>217</v>
       </c>
       <c r="P16" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -3900,7 +3902,7 @@
         <v>231</v>
       </c>
       <c r="P20" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
@@ -3946,7 +3948,7 @@
         <v>231</v>
       </c>
       <c r="P21" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
@@ -3981,11 +3983,11 @@
       <c r="K22" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L22" s="6" t="str">
-        <f>=IF(I22&lt;&gt;"",I22,IF(AND(G22&lt;&gt;"",H22&lt;&gt;""),G22*(1-H22/100),""))</f>
-      </c>
-      <c r="M22" s="6" t="str">
-        <f>=IF(J22&lt;&gt;"",J22,IF(AND(G22&lt;&gt;"",H22&lt;&gt;""),G22*(1+H22/100),""))</f>
+      <c r="L22" s="6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M22" s="6" t="n">
+        <v>0.027</v>
       </c>
       <c r="N22" s="5" t="s">
         <v>15</v>
@@ -3994,7 +3996,7 @@
         <v>237</v>
       </c>
       <c r="P22" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -4029,11 +4031,11 @@
       <c r="K23" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="L23" s="6" t="str">
-        <f>=IF(I23&lt;&gt;"",I23,IF(AND(G23&lt;&gt;"",H23&lt;&gt;""),G23*(1-H23/100),""))</f>
-      </c>
-      <c r="M23" s="6" t="str">
-        <f>=IF(J23&lt;&gt;"",J23,IF(AND(G23&lt;&gt;"",H23&lt;&gt;""),G23*(1+H23/100),""))</f>
+      <c r="L23" s="6" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="M23" s="6" t="n">
+        <v>0.017</v>
       </c>
       <c r="N23" s="5" t="s">
         <v>15</v>
@@ -4042,7 +4044,7 @@
         <v>240</v>
       </c>
       <c r="P23" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
@@ -4077,11 +4079,11 @@
       <c r="K24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="L24" s="6" t="str">
-        <f>=IF(I24&lt;&gt;"",I24,IF(AND(G24&lt;&gt;"",H24&lt;&gt;""),G24*(1-H24/100),""))</f>
-      </c>
-      <c r="M24" s="6" t="str">
-        <f>=IF(J24&lt;&gt;"",J24,IF(AND(G24&lt;&gt;"",H24&lt;&gt;""),G24*(1+H24/100),""))</f>
+      <c r="L24" s="6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M24" s="6" t="n">
+        <v>0.02</v>
       </c>
       <c r="N24" s="5" t="s">
         <v>15</v>
@@ -4090,7 +4092,7 @@
         <v>240</v>
       </c>
       <c r="P24" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -4125,11 +4127,11 @@
       <c r="K25" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L25" s="6" t="str">
-        <f>=IF(I25&lt;&gt;"",I25,IF(AND(G25&lt;&gt;"",H25&lt;&gt;""),G25*(1-H25/100),""))</f>
-      </c>
-      <c r="M25" s="6" t="str">
-        <f>=IF(J25&lt;&gt;"",J25,IF(AND(G25&lt;&gt;"",H25&lt;&gt;""),G25*(1+H25/100),""))</f>
+      <c r="L25" s="6" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="M25" s="6" t="n">
+        <v>0.31</v>
       </c>
       <c r="N25" s="5" t="s">
         <v>15</v>
@@ -4138,7 +4140,7 @@
         <v>240</v>
       </c>
       <c r="P25" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
@@ -4173,11 +4175,11 @@
       <c r="K26" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L26" s="6" t="str">
-        <f>=IF(I26&lt;&gt;"",I26,IF(AND(G26&lt;&gt;"",H26&lt;&gt;""),G26*(1-H26/100),""))</f>
-      </c>
-      <c r="M26" s="6" t="str">
-        <f>=IF(J26&lt;&gt;"",J26,IF(AND(G26&lt;&gt;"",H26&lt;&gt;""),G26*(1+H26/100),""))</f>
+      <c r="L26" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M26" s="6" t="n">
+        <v>0.73</v>
       </c>
       <c r="N26" s="5" t="s">
         <v>15</v>
@@ -4186,7 +4188,7 @@
         <v>240</v>
       </c>
       <c r="P26" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
@@ -4208,7 +4210,9 @@
       <c r="F27" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="G27" s="3"/>
+      <c r="G27" s="3" t="n">
+        <v>3.3</v>
+      </c>
       <c r="H27" s="3" t="n">
         <v>10</v>
       </c>
@@ -4217,11 +4221,11 @@
       <c r="K27" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="L27" s="6" t="str">
-        <f>=IF(I27&lt;&gt;"",I27,IF(AND(G27&lt;&gt;"",H27&lt;&gt;""),G27*(1-H27/100),""))</f>
-      </c>
-      <c r="M27" s="6" t="str">
-        <f>=IF(J27&lt;&gt;"",J27,IF(AND(G27&lt;&gt;"",H27&lt;&gt;""),G27*(1+H27/100),""))</f>
+      <c r="L27" s="6" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="M27" s="6" t="n">
+        <v>3.63</v>
       </c>
       <c r="N27" s="5" t="s">
         <v>15</v>
@@ -4230,7 +4234,7 @@
         <v>249</v>
       </c>
       <c r="P27" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
@@ -4276,7 +4280,7 @@
         <v>253</v>
       </c>
       <c r="P28" s="7" t="s">
-        <v>132</v>
+        <v>20</v>
       </c>
     </row>
     <row r="29">
@@ -4528,22 +4532,31 @@
       <c r="F34" t="s">
         <v>194</v>
       </c>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
+      <c r="G34" s="3" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I34" s="7"/>
       <c r="J34" s="7"/>
-      <c r="K34" s="4"/>
-      <c r="L34" s="6" t="str">
-        <f>=IF(I34&lt;&gt;"",I34,IF(AND(G34&lt;&gt;"",H34&lt;&gt;""),G34*(1-H34/100),""))</f>
-      </c>
-      <c r="M34" s="6" t="str">
-        <f>=IF(J34&lt;&gt;"",J34,IF(AND(G34&lt;&gt;"",H34&lt;&gt;""),G34*(1+H34/100),""))</f>
+      <c r="K34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="L34" s="6" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="M34" s="6" t="n">
+        <v>4.73</v>
       </c>
       <c r="N34" t="s">
         <v>15</v>
       </c>
       <c r="O34" t="s">
         <v>132</v>
+      </c>
+      <c r="P34" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="35">
@@ -4657,22 +4670,31 @@
       <c r="F37" t="s">
         <v>202</v>
       </c>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
+      <c r="G37" s="3" t="n">
+        <v>0.386</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>30</v>
+      </c>
       <c r="I37" s="7"/>
       <c r="J37" s="7"/>
-      <c r="K37" s="4"/>
-      <c r="L37" s="6" t="str">
-        <f>=IF(I37&lt;&gt;"",I37,IF(AND(G37&lt;&gt;"",H37&lt;&gt;""),G37*(1-H37/100),""))</f>
-      </c>
-      <c r="M37" s="6" t="str">
-        <f>=IF(J37&lt;&gt;"",J37,IF(AND(G37&lt;&gt;"",H37&lt;&gt;""),G37*(1+H37/100),""))</f>
+      <c r="K37" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L37" s="6" t="n">
+        <v>0.2702</v>
+      </c>
+      <c r="M37" s="6" t="n">
+        <v>0.5018</v>
       </c>
       <c r="N37" t="s">
         <v>15</v>
       </c>
       <c r="O37" t="s">
         <v>203</v>
+      </c>
+      <c r="P37" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="38">
@@ -4694,22 +4716,31 @@
       <c r="F38" t="s">
         <v>206</v>
       </c>
-      <c r="G38" s="3"/>
-      <c r="H38" s="3"/>
+      <c r="G38" s="3" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>30</v>
+      </c>
       <c r="I38" s="7"/>
       <c r="J38" s="7"/>
-      <c r="K38" s="4"/>
-      <c r="L38" s="6" t="str">
-        <f>=IF(I38&lt;&gt;"",I38,IF(AND(G38&lt;&gt;"",H38&lt;&gt;""),G38*(1-H38/100),""))</f>
-      </c>
-      <c r="M38" s="6" t="str">
-        <f>=IF(J38&lt;&gt;"",J38,IF(AND(G38&lt;&gt;"",H38&lt;&gt;""),G38*(1+H38/100),""))</f>
+      <c r="K38" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L38" s="6" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="M38" s="6" t="n">
+        <v>0.221</v>
       </c>
       <c r="N38" t="s">
         <v>15</v>
       </c>
       <c r="O38" t="s">
         <v>207</v>
+      </c>
+      <c r="P38" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="39">
@@ -4731,22 +4762,31 @@
       <c r="F39" t="s">
         <v>206</v>
       </c>
-      <c r="G39" s="3"/>
-      <c r="H39" s="3"/>
+      <c r="G39" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>30</v>
+      </c>
       <c r="I39" s="7"/>
       <c r="J39" s="7"/>
-      <c r="K39" s="4"/>
-      <c r="L39" s="6" t="str">
-        <f>=IF(I39&lt;&gt;"",I39,IF(AND(G39&lt;&gt;"",H39&lt;&gt;""),G39*(1-H39/100),""))</f>
-      </c>
-      <c r="M39" s="6" t="str">
-        <f>=IF(J39&lt;&gt;"",J39,IF(AND(G39&lt;&gt;"",H39&lt;&gt;""),G39*(1+H39/100),""))</f>
+      <c r="K39" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L39" s="6" t="n">
+        <v>0.56</v>
+      </c>
+      <c r="M39" s="6" t="n">
+        <v>1.04</v>
       </c>
       <c r="N39" t="s">
         <v>15</v>
       </c>
       <c r="O39" t="s">
         <v>210</v>
+      </c>
+      <c r="P39" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="40">
@@ -4768,22 +4808,31 @@
       <c r="F40" t="s">
         <v>206</v>
       </c>
-      <c r="G40" s="3"/>
-      <c r="H40" s="3"/>
+      <c r="G40" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I40" s="7"/>
       <c r="J40" s="7"/>
-      <c r="K40" s="4"/>
-      <c r="L40" s="6" t="str">
-        <f>=IF(I40&lt;&gt;"",I40,IF(AND(G40&lt;&gt;"",H40&lt;&gt;""),G40*(1-H40/100),""))</f>
-      </c>
-      <c r="M40" s="6" t="str">
-        <f>=IF(J40&lt;&gt;"",J40,IF(AND(G40&lt;&gt;"",H40&lt;&gt;""),G40*(1+H40/100),""))</f>
+      <c r="K40" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L40" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="M40" s="6" t="n">
+        <v>0.11</v>
       </c>
       <c r="N40" t="s">
         <v>15</v>
       </c>
       <c r="O40" t="s">
         <v>213</v>
+      </c>
+      <c r="P40" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="41">
@@ -4805,22 +4854,31 @@
       <c r="F41" t="s">
         <v>216</v>
       </c>
-      <c r="G41" s="3"/>
-      <c r="H41" s="3"/>
+      <c r="G41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>20</v>
+      </c>
       <c r="I41" s="7"/>
       <c r="J41" s="7"/>
-      <c r="K41" s="4"/>
-      <c r="L41" s="6" t="str">
-        <f>=IF(I41&lt;&gt;"",I41,IF(AND(G41&lt;&gt;"",H41&lt;&gt;""),G41*(1-H41/100),""))</f>
-      </c>
-      <c r="M41" s="6" t="str">
-        <f>=IF(J41&lt;&gt;"",J41,IF(AND(G41&lt;&gt;"",H41&lt;&gt;""),G41*(1+H41/100),""))</f>
+      <c r="K41" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="N41" t="s">
         <v>15</v>
       </c>
       <c r="O41" t="s">
         <v>217</v>
+      </c>
+      <c r="P41" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="42">
@@ -4980,22 +5038,31 @@
       <c r="F45" t="s">
         <v>230</v>
       </c>
-      <c r="G45" s="3"/>
-      <c r="H45" s="3"/>
+      <c r="G45" s="3" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="I45" s="7"/>
       <c r="J45" s="7"/>
-      <c r="K45" s="4"/>
-      <c r="L45" s="6" t="str">
-        <f>=IF(I45&lt;&gt;"",I45,IF(AND(G45&lt;&gt;"",H45&lt;&gt;""),G45*(1-H45/100),""))</f>
-      </c>
-      <c r="M45" s="6" t="str">
-        <f>=IF(J45&lt;&gt;"",J45,IF(AND(G45&lt;&gt;"",H45&lt;&gt;""),G45*(1+H45/100),""))</f>
+      <c r="K45" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L45" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M45" s="6" t="n">
+        <v>0.1</v>
       </c>
       <c r="N45" t="s">
         <v>15</v>
       </c>
       <c r="O45" t="s">
         <v>231</v>
+      </c>
+      <c r="P45" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="46">
@@ -5017,22 +5084,31 @@
       <c r="F46" t="s">
         <v>230</v>
       </c>
-      <c r="G46" s="3"/>
-      <c r="H46" s="3"/>
+      <c r="G46" s="3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="I46" s="7"/>
       <c r="J46" s="7"/>
-      <c r="K46" s="4"/>
-      <c r="L46" s="6" t="str">
-        <f>=IF(I46&lt;&gt;"",I46,IF(AND(G46&lt;&gt;"",H46&lt;&gt;""),G46*(1-H46/100),""))</f>
-      </c>
-      <c r="M46" s="6" t="str">
-        <f>=IF(J46&lt;&gt;"",J46,IF(AND(G46&lt;&gt;"",H46&lt;&gt;""),G46*(1+H46/100),""))</f>
+      <c r="K46" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L46" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M46" s="6" t="n">
+        <v>0.05</v>
       </c>
       <c r="N46" t="s">
         <v>15</v>
       </c>
       <c r="O46" t="s">
         <v>231</v>
+      </c>
+      <c r="P46" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="47">
@@ -5054,22 +5130,29 @@
       <c r="F47" t="s">
         <v>236</v>
       </c>
-      <c r="G47" s="3"/>
+      <c r="G47" s="3" t="n">
+        <v>0.006</v>
+      </c>
       <c r="H47" s="3"/>
       <c r="I47" s="7"/>
       <c r="J47" s="7"/>
-      <c r="K47" s="4"/>
-      <c r="L47" s="6" t="str">
-        <f>=IF(I47&lt;&gt;"",I47,IF(AND(G47&lt;&gt;"",H47&lt;&gt;""),G47*(1-H47/100),""))</f>
-      </c>
-      <c r="M47" s="6" t="str">
-        <f>=IF(J47&lt;&gt;"",J47,IF(AND(G47&lt;&gt;"",H47&lt;&gt;""),G47*(1+H47/100),""))</f>
+      <c r="K47" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L47" s="6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M47" s="6" t="n">
+        <v>0.027</v>
       </c>
       <c r="N47" t="s">
         <v>15</v>
       </c>
       <c r="O47" t="s">
         <v>237</v>
+      </c>
+      <c r="P47" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="48">
@@ -5091,22 +5174,29 @@
       <c r="F48" t="s">
         <v>236</v>
       </c>
-      <c r="G48" s="3"/>
+      <c r="G48" s="3" t="n">
+        <v>0.014</v>
+      </c>
       <c r="H48" s="3"/>
       <c r="I48" s="7"/>
       <c r="J48" s="7"/>
-      <c r="K48" s="4"/>
-      <c r="L48" s="6" t="str">
-        <f>=IF(I48&lt;&gt;"",I48,IF(AND(G48&lt;&gt;"",H48&lt;&gt;""),G48*(1-H48/100),""))</f>
-      </c>
-      <c r="M48" s="6" t="str">
-        <f>=IF(J48&lt;&gt;"",J48,IF(AND(G48&lt;&gt;"",H48&lt;&gt;""),G48*(1+H48/100),""))</f>
+      <c r="K48" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L48" s="6" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="M48" s="6" t="n">
+        <v>0.017</v>
       </c>
       <c r="N48" t="s">
         <v>15</v>
       </c>
       <c r="O48" t="s">
         <v>240</v>
+      </c>
+      <c r="P48" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="49">
@@ -5128,22 +5218,29 @@
       <c r="F49" t="s">
         <v>236</v>
       </c>
-      <c r="G49" s="3"/>
+      <c r="G49" s="3" t="n">
+        <v>0.011</v>
+      </c>
       <c r="H49" s="3"/>
       <c r="I49" s="7"/>
       <c r="J49" s="7"/>
-      <c r="K49" s="4"/>
-      <c r="L49" s="6" t="str">
-        <f>=IF(I49&lt;&gt;"",I49,IF(AND(G49&lt;&gt;"",H49&lt;&gt;""),G49*(1-H49/100),""))</f>
-      </c>
-      <c r="M49" s="6" t="str">
-        <f>=IF(J49&lt;&gt;"",J49,IF(AND(G49&lt;&gt;"",H49&lt;&gt;""),G49*(1+H49/100),""))</f>
+      <c r="K49" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L49" s="6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M49" s="6" t="n">
+        <v>0.02</v>
       </c>
       <c r="N49" t="s">
         <v>15</v>
       </c>
       <c r="O49" t="s">
         <v>240</v>
+      </c>
+      <c r="P49" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="50">
@@ -5165,22 +5262,29 @@
       <c r="F50" t="s">
         <v>230</v>
       </c>
-      <c r="G50" s="3"/>
+      <c r="G50" s="3" t="n">
+        <v>0.21</v>
+      </c>
       <c r="H50" s="3"/>
       <c r="I50" s="7"/>
       <c r="J50" s="7"/>
-      <c r="K50" s="4"/>
-      <c r="L50" s="6" t="str">
-        <f>=IF(I50&lt;&gt;"",I50,IF(AND(G50&lt;&gt;"",H50&lt;&gt;""),G50*(1-H50/100),""))</f>
-      </c>
-      <c r="M50" s="6" t="str">
-        <f>=IF(J50&lt;&gt;"",J50,IF(AND(G50&lt;&gt;"",H50&lt;&gt;""),G50*(1+H50/100),""))</f>
+      <c r="K50" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L50" s="6" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="M50" s="6" t="n">
+        <v>0.31</v>
       </c>
       <c r="N50" t="s">
         <v>15</v>
       </c>
       <c r="O50" t="s">
         <v>240</v>
+      </c>
+      <c r="P50" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="51">
@@ -5202,22 +5306,29 @@
       <c r="F51" t="s">
         <v>230</v>
       </c>
-      <c r="G51" s="3"/>
+      <c r="G51" s="3" t="n">
+        <v>0.24</v>
+      </c>
       <c r="H51" s="3"/>
       <c r="I51" s="7"/>
       <c r="J51" s="7"/>
-      <c r="K51" s="4"/>
-      <c r="L51" s="6" t="str">
-        <f>=IF(I51&lt;&gt;"",I51,IF(AND(G51&lt;&gt;"",H51&lt;&gt;""),G51*(1-H51/100),""))</f>
-      </c>
-      <c r="M51" s="6" t="str">
-        <f>=IF(J51&lt;&gt;"",J51,IF(AND(G51&lt;&gt;"",H51&lt;&gt;""),G51*(1+H51/100),""))</f>
+      <c r="K51" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L51" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M51" s="6" t="n">
+        <v>0.73</v>
       </c>
       <c r="N51" t="s">
         <v>15</v>
       </c>
       <c r="O51" t="s">
         <v>240</v>
+      </c>
+      <c r="P51" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="52">
@@ -5239,22 +5350,31 @@
       <c r="F52" t="s">
         <v>194</v>
       </c>
-      <c r="G52" s="3"/>
-      <c r="H52" s="3"/>
+      <c r="G52" s="3" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H52" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I52" s="7"/>
       <c r="J52" s="7"/>
-      <c r="K52" s="4"/>
-      <c r="L52" s="6" t="str">
-        <f>=IF(I52&lt;&gt;"",I52,IF(AND(G52&lt;&gt;"",H52&lt;&gt;""),G52*(1-H52/100),""))</f>
-      </c>
-      <c r="M52" s="6" t="str">
-        <f>=IF(J52&lt;&gt;"",J52,IF(AND(G52&lt;&gt;"",H52&lt;&gt;""),G52*(1+H52/100),""))</f>
+      <c r="K52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="L52" s="6" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="M52" s="6" t="n">
+        <v>3.63</v>
       </c>
       <c r="N52" t="s">
         <v>15</v>
       </c>
       <c r="O52" t="s">
         <v>249</v>
+      </c>
+      <c r="P52" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="53">
@@ -5276,22 +5396,31 @@
       <c r="F53" t="s">
         <v>252</v>
       </c>
-      <c r="G53" s="3"/>
-      <c r="H53" s="3"/>
+      <c r="G53" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H53" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="I53" s="7"/>
       <c r="J53" s="7"/>
-      <c r="K53" s="4"/>
-      <c r="L53" s="6" t="str">
-        <f>=IF(I53&lt;&gt;"",I53,IF(AND(G53&lt;&gt;"",H53&lt;&gt;""),G53*(1-H53/100),""))</f>
-      </c>
-      <c r="M53" s="6" t="str">
-        <f>=IF(J53&lt;&gt;"",J53,IF(AND(G53&lt;&gt;"",H53&lt;&gt;""),G53*(1+H53/100),""))</f>
+      <c r="K53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="L53" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M53" s="6" t="n">
+        <v>25</v>
       </c>
       <c r="N53" t="s">
         <v>15</v>
       </c>
       <c r="O53" t="s">
         <v>253</v>
+      </c>
+      <c r="P53" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="54">
@@ -5681,22 +5810,31 @@
       <c r="F62" t="s">
         <v>202</v>
       </c>
-      <c r="G62" s="3"/>
-      <c r="H62" s="3"/>
+      <c r="G62" s="3" t="n">
+        <v>0.386</v>
+      </c>
+      <c r="H62" s="3" t="n">
+        <v>30</v>
+      </c>
       <c r="I62" s="7"/>
       <c r="J62" s="7"/>
-      <c r="K62" s="4"/>
-      <c r="L62" s="6" t="str">
-        <f>=IF(I62&lt;&gt;"",I62,IF(AND(G62&lt;&gt;"",H62&lt;&gt;""),G62*(1-H62/100),""))</f>
-      </c>
-      <c r="M62" s="6" t="str">
-        <f>=IF(J62&lt;&gt;"",J62,IF(AND(G62&lt;&gt;"",H62&lt;&gt;""),G62*(1+H62/100),""))</f>
+      <c r="K62" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L62" s="6" t="n">
+        <v>0.2702</v>
+      </c>
+      <c r="M62" s="6" t="n">
+        <v>0.5018</v>
       </c>
       <c r="N62" t="s">
         <v>15</v>
       </c>
       <c r="O62" t="s">
         <v>203</v>
+      </c>
+      <c r="P62" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="63">
@@ -5718,22 +5856,31 @@
       <c r="F63" t="s">
         <v>206</v>
       </c>
-      <c r="G63" s="3"/>
-      <c r="H63" s="3"/>
+      <c r="G63" s="3" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H63" s="3" t="n">
+        <v>30</v>
+      </c>
       <c r="I63" s="7"/>
       <c r="J63" s="7"/>
-      <c r="K63" s="4"/>
-      <c r="L63" s="6" t="str">
-        <f>=IF(I63&lt;&gt;"",I63,IF(AND(G63&lt;&gt;"",H63&lt;&gt;""),G63*(1-H63/100),""))</f>
-      </c>
-      <c r="M63" s="6" t="str">
-        <f>=IF(J63&lt;&gt;"",J63,IF(AND(G63&lt;&gt;"",H63&lt;&gt;""),G63*(1+H63/100),""))</f>
+      <c r="K63" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L63" s="6" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="M63" s="6" t="n">
+        <v>0.221</v>
       </c>
       <c r="N63" t="s">
         <v>15</v>
       </c>
       <c r="O63" t="s">
         <v>207</v>
+      </c>
+      <c r="P63" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="64">
@@ -5755,22 +5902,31 @@
       <c r="F64" t="s">
         <v>206</v>
       </c>
-      <c r="G64" s="3"/>
-      <c r="H64" s="3"/>
+      <c r="G64" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H64" s="3" t="n">
+        <v>30</v>
+      </c>
       <c r="I64" s="7"/>
       <c r="J64" s="7"/>
-      <c r="K64" s="4"/>
-      <c r="L64" s="6" t="str">
-        <f>=IF(I64&lt;&gt;"",I64,IF(AND(G64&lt;&gt;"",H64&lt;&gt;""),G64*(1-H64/100),""))</f>
-      </c>
-      <c r="M64" s="6" t="str">
-        <f>=IF(J64&lt;&gt;"",J64,IF(AND(G64&lt;&gt;"",H64&lt;&gt;""),G64*(1+H64/100),""))</f>
+      <c r="K64" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L64" s="6" t="n">
+        <v>0.56</v>
+      </c>
+      <c r="M64" s="6" t="n">
+        <v>1.04</v>
       </c>
       <c r="N64" t="s">
         <v>15</v>
       </c>
       <c r="O64" t="s">
         <v>210</v>
+      </c>
+      <c r="P64" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="65">
@@ -5792,22 +5948,31 @@
       <c r="F65" t="s">
         <v>206</v>
       </c>
-      <c r="G65" s="3"/>
-      <c r="H65" s="3"/>
+      <c r="G65" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H65" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I65" s="7"/>
       <c r="J65" s="7"/>
-      <c r="K65" s="4"/>
-      <c r="L65" s="6" t="str">
-        <f>=IF(I65&lt;&gt;"",I65,IF(AND(G65&lt;&gt;"",H65&lt;&gt;""),G65*(1-H65/100),""))</f>
-      </c>
-      <c r="M65" s="6" t="str">
-        <f>=IF(J65&lt;&gt;"",J65,IF(AND(G65&lt;&gt;"",H65&lt;&gt;""),G65*(1+H65/100),""))</f>
+      <c r="K65" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L65" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="M65" s="6" t="n">
+        <v>0.11</v>
       </c>
       <c r="N65" t="s">
         <v>15</v>
       </c>
       <c r="O65" t="s">
         <v>213</v>
+      </c>
+      <c r="P65" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="66">
@@ -5829,22 +5994,31 @@
       <c r="F66" t="s">
         <v>216</v>
       </c>
-      <c r="G66" s="3"/>
-      <c r="H66" s="3"/>
+      <c r="G66" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" s="3" t="n">
+        <v>20</v>
+      </c>
       <c r="I66" s="7"/>
       <c r="J66" s="7"/>
-      <c r="K66" s="4"/>
-      <c r="L66" s="6" t="str">
-        <f>=IF(I66&lt;&gt;"",I66,IF(AND(G66&lt;&gt;"",H66&lt;&gt;""),G66*(1-H66/100),""))</f>
-      </c>
-      <c r="M66" s="6" t="str">
-        <f>=IF(J66&lt;&gt;"",J66,IF(AND(G66&lt;&gt;"",H66&lt;&gt;""),G66*(1+H66/100),""))</f>
+      <c r="K66" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L66" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M66" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="N66" t="s">
         <v>15</v>
       </c>
       <c r="O66" t="s">
         <v>217</v>
+      </c>
+      <c r="P66" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="67">
@@ -6004,22 +6178,31 @@
       <c r="F70" t="s">
         <v>230</v>
       </c>
-      <c r="G70" s="3"/>
-      <c r="H70" s="3"/>
+      <c r="G70" s="3" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H70" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="I70" s="7"/>
       <c r="J70" s="7"/>
-      <c r="K70" s="4"/>
-      <c r="L70" s="6" t="str">
-        <f>=IF(I70&lt;&gt;"",I70,IF(AND(G70&lt;&gt;"",H70&lt;&gt;""),G70*(1-H70/100),""))</f>
-      </c>
-      <c r="M70" s="6" t="str">
-        <f>=IF(J70&lt;&gt;"",J70,IF(AND(G70&lt;&gt;"",H70&lt;&gt;""),G70*(1+H70/100),""))</f>
+      <c r="K70" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L70" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M70" s="6" t="n">
+        <v>0.1</v>
       </c>
       <c r="N70" t="s">
         <v>15</v>
       </c>
       <c r="O70" t="s">
         <v>231</v>
+      </c>
+      <c r="P70" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="71">
@@ -6041,22 +6224,31 @@
       <c r="F71" t="s">
         <v>230</v>
       </c>
-      <c r="G71" s="3"/>
-      <c r="H71" s="3"/>
+      <c r="G71" s="3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H71" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="I71" s="7"/>
       <c r="J71" s="7"/>
-      <c r="K71" s="4"/>
-      <c r="L71" s="6" t="str">
-        <f>=IF(I71&lt;&gt;"",I71,IF(AND(G71&lt;&gt;"",H71&lt;&gt;""),G71*(1-H71/100),""))</f>
-      </c>
-      <c r="M71" s="6" t="str">
-        <f>=IF(J71&lt;&gt;"",J71,IF(AND(G71&lt;&gt;"",H71&lt;&gt;""),G71*(1+H71/100),""))</f>
+      <c r="K71" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L71" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M71" s="6" t="n">
+        <v>0.05</v>
       </c>
       <c r="N71" t="s">
         <v>15</v>
       </c>
       <c r="O71" t="s">
         <v>231</v>
+      </c>
+      <c r="P71" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="72">
@@ -6078,22 +6270,29 @@
       <c r="F72" t="s">
         <v>236</v>
       </c>
-      <c r="G72" s="3"/>
+      <c r="G72" s="3" t="n">
+        <v>0.006</v>
+      </c>
       <c r="H72" s="3"/>
       <c r="I72" s="7"/>
       <c r="J72" s="7"/>
-      <c r="K72" s="4"/>
-      <c r="L72" s="6" t="str">
-        <f>=IF(I72&lt;&gt;"",I72,IF(AND(G72&lt;&gt;"",H72&lt;&gt;""),G72*(1-H72/100),""))</f>
-      </c>
-      <c r="M72" s="6" t="str">
-        <f>=IF(J72&lt;&gt;"",J72,IF(AND(G72&lt;&gt;"",H72&lt;&gt;""),G72*(1+H72/100),""))</f>
+      <c r="K72" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L72" s="6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M72" s="6" t="n">
+        <v>0.027</v>
       </c>
       <c r="N72" t="s">
         <v>15</v>
       </c>
       <c r="O72" t="s">
         <v>237</v>
+      </c>
+      <c r="P72" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="73">
@@ -6115,22 +6314,29 @@
       <c r="F73" t="s">
         <v>236</v>
       </c>
-      <c r="G73" s="3"/>
+      <c r="G73" s="3" t="n">
+        <v>0.014</v>
+      </c>
       <c r="H73" s="3"/>
       <c r="I73" s="7"/>
       <c r="J73" s="7"/>
-      <c r="K73" s="4"/>
-      <c r="L73" s="6" t="str">
-        <f>=IF(I73&lt;&gt;"",I73,IF(AND(G73&lt;&gt;"",H73&lt;&gt;""),G73*(1-H73/100),""))</f>
-      </c>
-      <c r="M73" s="6" t="str">
-        <f>=IF(J73&lt;&gt;"",J73,IF(AND(G73&lt;&gt;"",H73&lt;&gt;""),G73*(1+H73/100),""))</f>
+      <c r="K73" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L73" s="6" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="M73" s="6" t="n">
+        <v>0.017</v>
       </c>
       <c r="N73" t="s">
         <v>15</v>
       </c>
       <c r="O73" t="s">
         <v>240</v>
+      </c>
+      <c r="P73" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="74">
@@ -6152,22 +6358,29 @@
       <c r="F74" t="s">
         <v>236</v>
       </c>
-      <c r="G74" s="3"/>
+      <c r="G74" s="3" t="n">
+        <v>0.011</v>
+      </c>
       <c r="H74" s="3"/>
       <c r="I74" s="7"/>
       <c r="J74" s="7"/>
-      <c r="K74" s="4"/>
-      <c r="L74" s="6" t="str">
-        <f>=IF(I74&lt;&gt;"",I74,IF(AND(G74&lt;&gt;"",H74&lt;&gt;""),G74*(1-H74/100),""))</f>
-      </c>
-      <c r="M74" s="6" t="str">
-        <f>=IF(J74&lt;&gt;"",J74,IF(AND(G74&lt;&gt;"",H74&lt;&gt;""),G74*(1+H74/100),""))</f>
+      <c r="K74" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L74" s="6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M74" s="6" t="n">
+        <v>0.02</v>
       </c>
       <c r="N74" t="s">
         <v>15</v>
       </c>
       <c r="O74" t="s">
         <v>240</v>
+      </c>
+      <c r="P74" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="75">
@@ -6189,22 +6402,29 @@
       <c r="F75" t="s">
         <v>230</v>
       </c>
-      <c r="G75" s="3"/>
+      <c r="G75" s="3" t="n">
+        <v>0.21</v>
+      </c>
       <c r="H75" s="3"/>
       <c r="I75" s="7"/>
       <c r="J75" s="7"/>
-      <c r="K75" s="4"/>
-      <c r="L75" s="6" t="str">
-        <f>=IF(I75&lt;&gt;"",I75,IF(AND(G75&lt;&gt;"",H75&lt;&gt;""),G75*(1-H75/100),""))</f>
-      </c>
-      <c r="M75" s="6" t="str">
-        <f>=IF(J75&lt;&gt;"",J75,IF(AND(G75&lt;&gt;"",H75&lt;&gt;""),G75*(1+H75/100),""))</f>
+      <c r="K75" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L75" s="6" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="M75" s="6" t="n">
+        <v>0.31</v>
       </c>
       <c r="N75" t="s">
         <v>15</v>
       </c>
       <c r="O75" t="s">
         <v>240</v>
+      </c>
+      <c r="P75" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="76">
@@ -6226,22 +6446,29 @@
       <c r="F76" t="s">
         <v>230</v>
       </c>
-      <c r="G76" s="3"/>
+      <c r="G76" s="3" t="n">
+        <v>0.24</v>
+      </c>
       <c r="H76" s="3"/>
       <c r="I76" s="7"/>
       <c r="J76" s="7"/>
-      <c r="K76" s="4"/>
-      <c r="L76" s="6" t="str">
-        <f>=IF(I76&lt;&gt;"",I76,IF(AND(G76&lt;&gt;"",H76&lt;&gt;""),G76*(1-H76/100),""))</f>
-      </c>
-      <c r="M76" s="6" t="str">
-        <f>=IF(J76&lt;&gt;"",J76,IF(AND(G76&lt;&gt;"",H76&lt;&gt;""),G76*(1+H76/100),""))</f>
+      <c r="K76" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L76" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M76" s="6" t="n">
+        <v>0.73</v>
       </c>
       <c r="N76" t="s">
         <v>15</v>
       </c>
       <c r="O76" t="s">
         <v>240</v>
+      </c>
+      <c r="P76" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="77">
@@ -6263,22 +6490,31 @@
       <c r="F77" t="s">
         <v>194</v>
       </c>
-      <c r="G77" s="3"/>
-      <c r="H77" s="3"/>
+      <c r="G77" s="3" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H77" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I77" s="7"/>
       <c r="J77" s="7"/>
-      <c r="K77" s="4"/>
-      <c r="L77" s="6" t="str">
-        <f>=IF(I77&lt;&gt;"",I77,IF(AND(G77&lt;&gt;"",H77&lt;&gt;""),G77*(1-H77/100),""))</f>
-      </c>
-      <c r="M77" s="6" t="str">
-        <f>=IF(J77&lt;&gt;"",J77,IF(AND(G77&lt;&gt;"",H77&lt;&gt;""),G77*(1+H77/100),""))</f>
+      <c r="K77" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="L77" s="6" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="M77" s="6" t="n">
+        <v>3.63</v>
       </c>
       <c r="N77" t="s">
         <v>15</v>
       </c>
       <c r="O77" t="s">
         <v>249</v>
+      </c>
+      <c r="P77" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="78">
@@ -6300,22 +6536,31 @@
       <c r="F78" t="s">
         <v>252</v>
       </c>
-      <c r="G78" s="3"/>
-      <c r="H78" s="3"/>
+      <c r="G78" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H78" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="I78" s="7"/>
       <c r="J78" s="7"/>
-      <c r="K78" s="4"/>
-      <c r="L78" s="6" t="str">
-        <f>=IF(I78&lt;&gt;"",I78,IF(AND(G78&lt;&gt;"",H78&lt;&gt;""),G78*(1-H78/100),""))</f>
-      </c>
-      <c r="M78" s="6" t="str">
-        <f>=IF(J78&lt;&gt;"",J78,IF(AND(G78&lt;&gt;"",H78&lt;&gt;""),G78*(1+H78/100),""))</f>
+      <c r="K78" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="L78" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M78" s="6" t="n">
+        <v>25</v>
       </c>
       <c r="N78" t="s">
         <v>15</v>
       </c>
       <c r="O78" t="s">
         <v>253</v>
+      </c>
+      <c r="P78" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="79">
@@ -6567,22 +6812,31 @@
       <c r="F84" t="s">
         <v>194</v>
       </c>
-      <c r="G84" s="3"/>
-      <c r="H84" s="3"/>
+      <c r="G84" s="3" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I84" s="7"/>
       <c r="J84" s="7"/>
-      <c r="K84" s="4"/>
-      <c r="L84" s="6" t="str">
-        <f>=IF(I84&lt;&gt;"",I84,IF(AND(G84&lt;&gt;"",H84&lt;&gt;""),G84*(1-H84/100),""))</f>
-      </c>
-      <c r="M84" s="6" t="str">
-        <f>=IF(J84&lt;&gt;"",J84,IF(AND(G84&lt;&gt;"",H84&lt;&gt;""),G84*(1+H84/100),""))</f>
+      <c r="K84" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="L84" s="6" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="M84" s="6" t="n">
+        <v>4.73</v>
       </c>
       <c r="N84" t="s">
         <v>15</v>
       </c>
       <c r="O84" t="s">
         <v>132</v>
+      </c>
+      <c r="P84" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="85">
@@ -6696,22 +6950,31 @@
       <c r="F87" t="s">
         <v>202</v>
       </c>
-      <c r="G87" s="3"/>
-      <c r="H87" s="3"/>
+      <c r="G87" s="3" t="n">
+        <v>0.386</v>
+      </c>
+      <c r="H87" s="3" t="n">
+        <v>30</v>
+      </c>
       <c r="I87" s="7"/>
       <c r="J87" s="7"/>
-      <c r="K87" s="4"/>
-      <c r="L87" s="6" t="str">
-        <f>=IF(I87&lt;&gt;"",I87,IF(AND(G87&lt;&gt;"",H87&lt;&gt;""),G87*(1-H87/100),""))</f>
-      </c>
-      <c r="M87" s="6" t="str">
-        <f>=IF(J87&lt;&gt;"",J87,IF(AND(G87&lt;&gt;"",H87&lt;&gt;""),G87*(1+H87/100),""))</f>
+      <c r="K87" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L87" s="6" t="n">
+        <v>0.2702</v>
+      </c>
+      <c r="M87" s="6" t="n">
+        <v>0.5018</v>
       </c>
       <c r="N87" t="s">
         <v>15</v>
       </c>
       <c r="O87" t="s">
         <v>203</v>
+      </c>
+      <c r="P87" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="88">
@@ -6733,22 +6996,31 @@
       <c r="F88" t="s">
         <v>206</v>
       </c>
-      <c r="G88" s="3"/>
-      <c r="H88" s="3"/>
+      <c r="G88" s="3" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H88" s="3" t="n">
+        <v>30</v>
+      </c>
       <c r="I88" s="7"/>
       <c r="J88" s="7"/>
-      <c r="K88" s="4"/>
-      <c r="L88" s="6" t="str">
-        <f>=IF(I88&lt;&gt;"",I88,IF(AND(G88&lt;&gt;"",H88&lt;&gt;""),G88*(1-H88/100),""))</f>
-      </c>
-      <c r="M88" s="6" t="str">
-        <f>=IF(J88&lt;&gt;"",J88,IF(AND(G88&lt;&gt;"",H88&lt;&gt;""),G88*(1+H88/100),""))</f>
+      <c r="K88" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L88" s="6" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="M88" s="6" t="n">
+        <v>0.221</v>
       </c>
       <c r="N88" t="s">
         <v>15</v>
       </c>
       <c r="O88" t="s">
         <v>207</v>
+      </c>
+      <c r="P88" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="89">
@@ -6770,22 +7042,31 @@
       <c r="F89" t="s">
         <v>206</v>
       </c>
-      <c r="G89" s="3"/>
-      <c r="H89" s="3"/>
+      <c r="G89" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>30</v>
+      </c>
       <c r="I89" s="7"/>
       <c r="J89" s="7"/>
-      <c r="K89" s="4"/>
-      <c r="L89" s="6" t="str">
-        <f>=IF(I89&lt;&gt;"",I89,IF(AND(G89&lt;&gt;"",H89&lt;&gt;""),G89*(1-H89/100),""))</f>
-      </c>
-      <c r="M89" s="6" t="str">
-        <f>=IF(J89&lt;&gt;"",J89,IF(AND(G89&lt;&gt;"",H89&lt;&gt;""),G89*(1+H89/100),""))</f>
+      <c r="K89" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L89" s="6" t="n">
+        <v>0.56</v>
+      </c>
+      <c r="M89" s="6" t="n">
+        <v>1.04</v>
       </c>
       <c r="N89" t="s">
         <v>15</v>
       </c>
       <c r="O89" t="s">
         <v>210</v>
+      </c>
+      <c r="P89" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="90">
@@ -6807,22 +7088,31 @@
       <c r="F90" t="s">
         <v>206</v>
       </c>
-      <c r="G90" s="3"/>
-      <c r="H90" s="3"/>
+      <c r="G90" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H90" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I90" s="7"/>
       <c r="J90" s="7"/>
-      <c r="K90" s="4"/>
-      <c r="L90" s="6" t="str">
-        <f>=IF(I90&lt;&gt;"",I90,IF(AND(G90&lt;&gt;"",H90&lt;&gt;""),G90*(1-H90/100),""))</f>
-      </c>
-      <c r="M90" s="6" t="str">
-        <f>=IF(J90&lt;&gt;"",J90,IF(AND(G90&lt;&gt;"",H90&lt;&gt;""),G90*(1+H90/100),""))</f>
+      <c r="K90" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L90" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="M90" s="6" t="n">
+        <v>0.11</v>
       </c>
       <c r="N90" t="s">
         <v>15</v>
       </c>
       <c r="O90" t="s">
         <v>213</v>
+      </c>
+      <c r="P90" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="91">
@@ -7028,22 +7318,31 @@
       <c r="F95" t="s">
         <v>230</v>
       </c>
-      <c r="G95" s="3"/>
-      <c r="H95" s="3"/>
+      <c r="G95" s="3" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H95" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="I95" s="7"/>
       <c r="J95" s="7"/>
-      <c r="K95" s="4"/>
-      <c r="L95" s="6" t="str">
-        <f>=IF(I95&lt;&gt;"",I95,IF(AND(G95&lt;&gt;"",H95&lt;&gt;""),G95*(1-H95/100),""))</f>
-      </c>
-      <c r="M95" s="6" t="str">
-        <f>=IF(J95&lt;&gt;"",J95,IF(AND(G95&lt;&gt;"",H95&lt;&gt;""),G95*(1+H95/100),""))</f>
+      <c r="K95" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L95" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M95" s="6" t="n">
+        <v>0.1</v>
       </c>
       <c r="N95" t="s">
         <v>15</v>
       </c>
       <c r="O95" t="s">
         <v>231</v>
+      </c>
+      <c r="P95" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="96">
@@ -7065,22 +7364,31 @@
       <c r="F96" t="s">
         <v>230</v>
       </c>
-      <c r="G96" s="3"/>
-      <c r="H96" s="3"/>
+      <c r="G96" s="3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H96" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="I96" s="7"/>
       <c r="J96" s="7"/>
-      <c r="K96" s="4"/>
-      <c r="L96" s="6" t="str">
-        <f>=IF(I96&lt;&gt;"",I96,IF(AND(G96&lt;&gt;"",H96&lt;&gt;""),G96*(1-H96/100),""))</f>
-      </c>
-      <c r="M96" s="6" t="str">
-        <f>=IF(J96&lt;&gt;"",J96,IF(AND(G96&lt;&gt;"",H96&lt;&gt;""),G96*(1+H96/100),""))</f>
+      <c r="K96" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L96" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M96" s="6" t="n">
+        <v>0.05</v>
       </c>
       <c r="N96" t="s">
         <v>15</v>
       </c>
       <c r="O96" t="s">
         <v>231</v>
+      </c>
+      <c r="P96" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="97">
@@ -7102,22 +7410,29 @@
       <c r="F97" t="s">
         <v>236</v>
       </c>
-      <c r="G97" s="3"/>
+      <c r="G97" s="3" t="n">
+        <v>0.006</v>
+      </c>
       <c r="H97" s="3"/>
       <c r="I97" s="7"/>
       <c r="J97" s="7"/>
-      <c r="K97" s="4"/>
-      <c r="L97" s="6" t="str">
-        <f>=IF(I97&lt;&gt;"",I97,IF(AND(G97&lt;&gt;"",H97&lt;&gt;""),G97*(1-H97/100),""))</f>
-      </c>
-      <c r="M97" s="6" t="str">
-        <f>=IF(J97&lt;&gt;"",J97,IF(AND(G97&lt;&gt;"",H97&lt;&gt;""),G97*(1+H97/100),""))</f>
+      <c r="K97" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L97" s="6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M97" s="6" t="n">
+        <v>0.027</v>
       </c>
       <c r="N97" t="s">
         <v>15</v>
       </c>
       <c r="O97" t="s">
         <v>237</v>
+      </c>
+      <c r="P97" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="98">
@@ -7139,22 +7454,29 @@
       <c r="F98" t="s">
         <v>236</v>
       </c>
-      <c r="G98" s="3"/>
+      <c r="G98" s="3" t="n">
+        <v>0.014</v>
+      </c>
       <c r="H98" s="3"/>
       <c r="I98" s="7"/>
       <c r="J98" s="7"/>
-      <c r="K98" s="4"/>
-      <c r="L98" s="6" t="str">
-        <f>=IF(I98&lt;&gt;"",I98,IF(AND(G98&lt;&gt;"",H98&lt;&gt;""),G98*(1-H98/100),""))</f>
-      </c>
-      <c r="M98" s="6" t="str">
-        <f>=IF(J98&lt;&gt;"",J98,IF(AND(G98&lt;&gt;"",H98&lt;&gt;""),G98*(1+H98/100),""))</f>
+      <c r="K98" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L98" s="6" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="M98" s="6" t="n">
+        <v>0.017</v>
       </c>
       <c r="N98" t="s">
         <v>15</v>
       </c>
       <c r="O98" t="s">
         <v>240</v>
+      </c>
+      <c r="P98" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="99">
@@ -7176,22 +7498,29 @@
       <c r="F99" t="s">
         <v>236</v>
       </c>
-      <c r="G99" s="3"/>
+      <c r="G99" s="3" t="n">
+        <v>0.011</v>
+      </c>
       <c r="H99" s="3"/>
       <c r="I99" s="7"/>
       <c r="J99" s="7"/>
-      <c r="K99" s="4"/>
-      <c r="L99" s="6" t="str">
-        <f>=IF(I99&lt;&gt;"",I99,IF(AND(G99&lt;&gt;"",H99&lt;&gt;""),G99*(1-H99/100),""))</f>
-      </c>
-      <c r="M99" s="6" t="str">
-        <f>=IF(J99&lt;&gt;"",J99,IF(AND(G99&lt;&gt;"",H99&lt;&gt;""),G99*(1+H99/100),""))</f>
+      <c r="K99" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L99" s="6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M99" s="6" t="n">
+        <v>0.02</v>
       </c>
       <c r="N99" t="s">
         <v>15</v>
       </c>
       <c r="O99" t="s">
         <v>240</v>
+      </c>
+      <c r="P99" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="100">
@@ -7213,22 +7542,29 @@
       <c r="F100" t="s">
         <v>230</v>
       </c>
-      <c r="G100" s="3"/>
+      <c r="G100" s="3" t="n">
+        <v>0.21</v>
+      </c>
       <c r="H100" s="3"/>
       <c r="I100" s="7"/>
       <c r="J100" s="7"/>
-      <c r="K100" s="4"/>
-      <c r="L100" s="6" t="str">
-        <f>=IF(I100&lt;&gt;"",I100,IF(AND(G100&lt;&gt;"",H100&lt;&gt;""),G100*(1-H100/100),""))</f>
-      </c>
-      <c r="M100" s="6" t="str">
-        <f>=IF(J100&lt;&gt;"",J100,IF(AND(G100&lt;&gt;"",H100&lt;&gt;""),G100*(1+H100/100),""))</f>
+      <c r="K100" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L100" s="6" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="M100" s="6" t="n">
+        <v>0.31</v>
       </c>
       <c r="N100" t="s">
         <v>15</v>
       </c>
       <c r="O100" t="s">
         <v>240</v>
+      </c>
+      <c r="P100" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="101">
@@ -7250,22 +7586,29 @@
       <c r="F101" t="s">
         <v>230</v>
       </c>
-      <c r="G101" s="3"/>
+      <c r="G101" s="3" t="n">
+        <v>0.24</v>
+      </c>
       <c r="H101" s="3"/>
       <c r="I101" s="7"/>
       <c r="J101" s="7"/>
-      <c r="K101" s="4"/>
-      <c r="L101" s="6" t="str">
-        <f>=IF(I101&lt;&gt;"",I101,IF(AND(G101&lt;&gt;"",H101&lt;&gt;""),G101*(1-H101/100),""))</f>
-      </c>
-      <c r="M101" s="6" t="str">
-        <f>=IF(J101&lt;&gt;"",J101,IF(AND(G101&lt;&gt;"",H101&lt;&gt;""),G101*(1+H101/100),""))</f>
+      <c r="K101" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="L101" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M101" s="6" t="n">
+        <v>0.73</v>
       </c>
       <c r="N101" t="s">
         <v>15</v>
       </c>
       <c r="O101" t="s">
         <v>240</v>
+      </c>
+      <c r="P101" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="102">
@@ -7287,22 +7630,31 @@
       <c r="F102" t="s">
         <v>194</v>
       </c>
-      <c r="G102" s="3"/>
-      <c r="H102" s="3"/>
+      <c r="G102" s="3" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H102" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I102" s="7"/>
       <c r="J102" s="7"/>
-      <c r="K102" s="4"/>
-      <c r="L102" s="6" t="str">
-        <f>=IF(I102&lt;&gt;"",I102,IF(AND(G102&lt;&gt;"",H102&lt;&gt;""),G102*(1-H102/100),""))</f>
-      </c>
-      <c r="M102" s="6" t="str">
-        <f>=IF(J102&lt;&gt;"",J102,IF(AND(G102&lt;&gt;"",H102&lt;&gt;""),G102*(1+H102/100),""))</f>
+      <c r="K102" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="L102" s="6" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="M102" s="6" t="n">
+        <v>3.63</v>
       </c>
       <c r="N102" t="s">
         <v>15</v>
       </c>
       <c r="O102" t="s">
         <v>249</v>
+      </c>
+      <c r="P102" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="103">
@@ -7324,22 +7676,31 @@
       <c r="F103" t="s">
         <v>252</v>
       </c>
-      <c r="G103" s="3"/>
-      <c r="H103" s="3"/>
+      <c r="G103" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H103" s="3" t="n">
+        <v>25</v>
+      </c>
       <c r="I103" s="7"/>
       <c r="J103" s="7"/>
-      <c r="K103" s="4"/>
-      <c r="L103" s="6" t="str">
-        <f>=IF(I103&lt;&gt;"",I103,IF(AND(G103&lt;&gt;"",H103&lt;&gt;""),G103*(1-H103/100),""))</f>
-      </c>
-      <c r="M103" s="6" t="str">
-        <f>=IF(J103&lt;&gt;"",J103,IF(AND(G103&lt;&gt;"",H103&lt;&gt;""),G103*(1+H103/100),""))</f>
+      <c r="K103" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="L103" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M103" s="6" t="n">
+        <v>25</v>
       </c>
       <c r="N103" t="s">
         <v>15</v>
       </c>
       <c r="O103" t="s">
         <v>253</v>
+      </c>
+      <c r="P103" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="104">
@@ -14935,13 +15296,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{840FDCEA-16A1-46AA-BF4A-29CF784E0B78}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD71A8D8-CBC8-48CC-8EDA-8DB1144BC89C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D72F50B9-E898-4594-AA79-CA7CD3A641D7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A80BCE90-8273-4A7C-801A-CF59BFD387FE}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{311D2BC6-7403-4009-AC34-8815B0C1E156}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{88822FF9-35C9-46E0-BD6A-983A79083E09}"/>
 </file>
</xml_diff>